<commit_message>
Weigh-in Form: Sync second sheet
</commit_message>
<xml_diff>
--- a/local/templates/weighin/WeighInForm.xlsx
+++ b/local/templates/weighin/WeighInForm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/scottgonzalez/Projects/Misc/usaw-owlcms/local/templates/weighin/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{23236522-88C7-8E49-A4C3-C802199A1981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3CC92289-C33C-BA4F-BC43-86C3A22E21E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="20520" yWindow="2600" windowWidth="39500" windowHeight="23500" xr2:uid="{295DEE46-55CB-FD4C-B22D-54961E31048E}"/>
   </bookViews>
@@ -138,7 +138,7 @@
     <author>Scott Gonzalez</author>
   </authors>
   <commentList>
-    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{5B576708-074F-5F4A-B4E9-E666136A2D22}">
+    <comment ref="A1" authorId="0" shapeId="0" xr:uid="{C16ACF1E-49F8-FF4E-947A-C84ACB213E56}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{53C2706A-84FB-A747-900E-08C08E38A7CD}">
+    <comment ref="A7" authorId="0" shapeId="0" xr:uid="{6EF16F77-7990-774D-8942-E9C12C8E4969}">
       <text>
         <r>
           <rPr>
@@ -229,7 +229,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="32">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="31">
   <si>
     <t>${competition.competitionName}</t>
   </si>
@@ -286,9 +286,6 @@
   </si>
   <si>
     <t>Gndr</t>
-  </si>
-  <si>
-    <t>Session ${session.name} - ${session.ageGroupInfo.0.formattedRange}</t>
   </si>
   <si>
     <t>Team</t>
@@ -439,7 +436,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -482,24 +479,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <fill>
         <patternFill>
@@ -508,29 +492,6 @@
       </fill>
     </dxf>
     <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
       <fill>
         <patternFill>
           <bgColor rgb="FFFFC7CE"/>
@@ -919,7 +880,7 @@
     </row>
     <row r="3" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -996,7 +957,7 @@
         <v>6</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>7</v>
@@ -1013,37 +974,37 @@
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1132,21 +1093,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="31" x14ac:dyDescent="0.35">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="15"/>
+      <c r="G1" s="15"/>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15"/>
+      <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" s="2"/>
@@ -1165,7 +1126,7 @@
     </row>
     <row r="3" spans="1:13" ht="24" x14ac:dyDescent="0.3">
       <c r="A3" s="11" t="s">
-        <v>19</v>
+        <v>30</v>
       </c>
       <c r="B3" s="11"/>
       <c r="C3" s="11"/>
@@ -1242,7 +1203,7 @@
         <v>6</v>
       </c>
       <c r="I6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="J6" s="3" t="s">
         <v>7</v>
@@ -1259,37 +1220,37 @@
     </row>
     <row r="7" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="B7" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="B7" s="7" t="s">
+      <c r="C7" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="C7" s="7" t="s">
+      <c r="D7" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="F7" s="6" t="s">
+      <c r="G7" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G7" s="5" t="s">
+      <c r="H7" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="I7" s="10" t="s">
         <v>28</v>
-      </c>
-      <c r="I7" s="10" t="s">
-        <v>29</v>
       </c>
       <c r="J7" s="5"/>
       <c r="K7" s="5"/>
       <c r="L7" s="5"/>
       <c r="M7" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.2">
@@ -1347,8 +1308,8 @@
     <mergeCell ref="I9:M9"/>
   </mergeCells>
   <conditionalFormatting sqref="F7">
-    <cfRule type="expression" dxfId="2" priority="1">
-      <formula>DATEDIF(F7, $A$4, "Y") &lt; 18</formula>
+    <cfRule type="cellIs" dxfId="0" priority="1" stopIfTrue="1" operator="greaterThan">
+      <formula>DATE(YEAR(A4) - 18, MONTH(A4), DAY(A4))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>